<commit_message>
add: assignment 3 plot 2 data
</commit_message>
<xml_diff>
--- a/02_activities/assignments/a3_plot2.xlsx
+++ b/02_activities/assignments/a3_plot2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vivianschu/repos/DSI/visualization/02_activities/assignments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F75B00-B5BC-6F40-9F1E-9AFD400105E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3135B4-D41B-6344-99AD-9A677F728DD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -805,7 +805,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Weekly E. coli Levels at Selected Toronto Beaches — Summer 2023</a:t>
+              <a:t>Weekly E. coli Levels at Selected Toronto Beaches - Summer 2023</a:t>
             </a:r>
           </a:p>
         </c:rich>

</xml_diff>